<commit_message>
feat: Redesign ToxiLingo UI featuring Mascot Peach, Speech Bubble, Question Box & Glowing Orb
</commit_message>
<xml_diff>
--- a/toxilingo_50_scripts.xlsx
+++ b/toxilingo_50_scripts.xlsx
@@ -455,7 +455,7 @@
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
@@ -526,7 +526,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Como culo? You eat ass? No wonder your breath smells like shit!</t>
+          <t>Como culo? You eat ass? ... HAHAHAHAHA! EWWWW! No wonder your breath smells like shit!</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -568,7 +568,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Yo como pies! You said I eat feet! Please, can you eat mine perrita?</t>
+          <t>Yo como pies! You said I eat feet! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Please, can you eat mine perrita?</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Mi coochie huele a huevos! Go wash your pussy pendeja!</t>
+          <t>Mi coochie huele a huevos! ... HAHAHAHAHA! EWWWW! Go wash your pussy pendeja!</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Dame el choco-ano tía! Congrats gringo, you just asked the waitress to eat her asshole with cheese!</t>
+          <t>Dame el choco-ano tía! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Congrats gringo, you just asked the waitress to eat her asshole with cheese!</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Slang / Insult</t>
+          <t>Medellin Slang / Insult</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Soy un gonorrea de primera! Perfect, now everyone knows you are a walking venereal disease!</t>
+          <t>Soy un gonorrea de primera! ... HAHAHAHAHA! EWWWW! Perfect, now everyone knows you are a walking venereal disease!</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Me encanta la verga en ensalada! Outstanding, you just declared your love for raw dick in your salad!</t>
+          <t>Me encanta la verga en ensalada! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Outstanding, you just declared your love for raw dick in your salad!</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -778,7 +778,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Tienes ojos de perra con rabia! Aww, telling her she has eyes of a rabid bitch is so romantic!</t>
+          <t>Tienes ojos de perra con rabia! ... HAHAHAHAHA! EWWWW! Aww, telling her she has eyes of a rabid bitch is so romantic!</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Estoy embarazada! Wow congrats bro, a gringo guy getting pregnant is a medical miracle!</t>
+          <t>Estoy embarazada! ... OH MY GOD!! HAHAHAHAHA! Congrats bro, a gringo guy getting pregnant is a medical miracle!</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Llévame al bicho cabrón! Great job, you just asked a scary local taxi driver to take you by his dick!</t>
+          <t>Llévame al bicho cabrón! ... HAHAHAHAHA! EWWWW! Great job, you just asked a scary local taxi driver to take you by his dick!</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -904,7 +904,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Soy retrasado mental no me peguen! Exactly right, begging locals not to beat you up for being stupid!</t>
+          <t>Soy retrasado mental no me peguen! ... OH MY GOD!! HAHAHAHAHA! Exactly right, begging locals not to beat you up for being stupid!</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Déjame manosear tu papaya mamacita! Perfect, sexual harassment charges in 3... 2... 1...</t>
+          <t>Déjame manosear tu papaya mamacita! ... HAHAHAHAHA! EWWWW! Sexual harassment charges in three... two... one!</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Parezco un chimpancé bañado! Spot on, you look like a freshly washed gorilla!</t>
+          <t>Parezco un chimpancé bañado! ... OH MY GOD!! HAHAHAHAHA! Spot on, you look like a freshly washed gorilla!</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Me duele el culo de tanto azotar! Wow, bragging about getting your ass clapped too hard!</t>
+          <t>Me duele el culo de tanto azotar! ... HAHAHAHAHA! EWWWW! Bragging about getting your ass clapped too hard!</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Dónde hay prepagos baratas socio? Nice! You just asked a random police officer where to buy cheap prostitutes!</t>
+          <t>Dónde hay prepagos baratas socio? ... OH MY GOD!! HAHAHAHAHA! EWWWW! You just asked a random police officer where to buy cheap prostitutes!</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Me chupo mi propia chocha! Incredible, claiming you can lick your own vagina!</t>
+          <t>Me chupo mi propia chocha! ... HAHAHAHAHA! EWWWW! Incredible, claiming you can lick your own vagina!</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Esta mierda es comestible milagro! Complimenting the chef that his shit is surprisingly edible!</t>
+          <t>Esta mierda es comestible milagro! ... OH MY GOD!! HAHAHAHAHA! Complimenting the chef that his shit is surprisingly edible!</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Estoy más caliente que una perra en celo! Beautiful, telling locals you are horny like a bitch in heat!</t>
+          <t>Estoy más caliente que una perra en celo! ... HAHAHAHAHA! EWWWW! Beautiful, telling locals you are horny like a bitch in heat!</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Soy tacaño y podrido téngame lástima! Asking for mercy because you are a rotten cheapskate!</t>
+          <t>Soy tacaño y podrido téngame lástima! ... OH MY GOD!! HAHAHAHAHA! Asking for mercy because you are a rotten cheapskate!</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Dame leche de tu manguera papi! Asking the bartender to feed you milk straight from his hose!</t>
+          <t>Dame leche de tu manguera papi! ... HAHAHAHAHA! EWWWW! Asking the bartender to feed you milk straight from his hose!</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1324,7 +1324,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Inyecto esteroides y sigo fofo! Telling everyone at the gym you inject juice and stay soft!</t>
+          <t>Inyecto esteroides y sigo fofo! ... OH MY GOD!! HAHAHAHAHA! Telling everyone at the gym you inject juice and stay soft!</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1366,7 +1366,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Ketsu wo nameasete kudasai! Congrats otaku, you just begged a Yakuza boss to let you lick his ass!</t>
+          <t>Ketsu wo nameasete kudasai! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Congrats otaku, you just begged a Yakuza boss to let you lick his ass!</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Ore no baka chinchin wo miro! Perfect, screaming 'look at my stupid penis' at a stranger!</t>
+          <t>Ore no baka chinchin wo miro! ... HAHAHAHAHA! EWWWW! Perfect, screaming 'look at my stupid penis' at a stranger!</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Kono shiru wa opai no aji ga suru! Telling the old chef his ramen tastes like breast milk!</t>
+          <t>Kono shiru wa opai no aji ga suru! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Telling the old chef his ramen tastes like breast milk!</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Eigo hanase baka gaijin domo! Shouting 'speak English you stupid foreigner pigs!'</t>
+          <t>Eigo hanase baka gaijin domo! ... HAHAHAHAHA! Shouting 'speak English you stupid foreigner pigs!'</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -1534,7 +1534,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>O-kyaku sama noパンツ wo kudasai! Asking the cute maid to hand over her underwear!</t>
+          <t>O-kyaku sama no pantsu wo kudasai! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Asking the cute maid to hand over her underwear!</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1576,7 +1576,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Koko de seppuku shimasu! Informing the cab driver you will commit ritual suicide right here!</t>
+          <t>Koko de seppuku shimasu! ... HAHAHAHAHA! Informing the cab driver you will commit ritual suicide right here!</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Gochisousama! Now pay double because you sounded like a samurai from 1500!</t>
+          <t>Gochisousama! ... OH MY GOD!! HAHAHAHAHA! Now pay double because you sounded like a samurai from 1500!</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Hadaka de chinchin dance ga taiketsu! Inviting elderly locals to a naked penis dance duel!</t>
+          <t>Hadaka de chinchin dance ga taiketsu! ... HAHAHAHAHA! EWWWW! Inviting elderly locals to a naked penis dance duel!</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Chikan ga tatakatte iru! Screaming 'the molesters are fighting each other!' on train</t>
+          <t>Chikan ga tatakatte iru! ... OH MY GOD!! HAHAHAHAHA! Screaming 'the molesters are fighting each other!' on the subway!</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Neko no kintama sugoi! Praising the magnificence of a cat's testicles!</t>
+          <t>Neko no kintama sugoi! ... HAHAHAHAHA! EWWWW! Praising the magnificence of a cat's testicles!</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1786,7 +1786,7 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>HALT MAUL UND ARBEITE SCHWEIN! Shouting 'SHUT UP AND WORK YOU SWINE!' at 7 AM!</t>
+          <t>HALT MAUL UND ARBEITE SCHWEIN! ... OH MY GOD!! HAHAHAHAHA! Shouting 'SHUT UP AND WORK YOU SWINE!' at 7 AM!</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1828,7 +1828,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Ein Bier und spritz mir ins Gesicht! Ordering one beer with a side of facial cumshot!</t>
+          <t>Ein Bier und spritz mir ins Gesicht! ... HAHAHAHAHA! EWWWW! Ordering one beer with a side of facial cumshot!</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -1870,7 +1870,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Ich möchte deine Oma essen! Asking the baker if you can eat his grandmother!</t>
+          <t>Ich möchte deine Oma essen! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Asking the baker if you can eat his grandmother!</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Ich bin ein illegaler Kartoffelkopf! Declaring yourself an illegal potato head!</t>
+          <t>Ich bin ein illegaler Kartoffelkopf! ... HAHAHAHAHA! Declaring yourself an illegal potato head!</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Ich stecke Wurst in meine Ritze! Telling the butcher you shove sausages up your crack!</t>
+          <t>Ich stecke Wurst in meine Ritze! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Telling the butcher you shove sausages up your crack!</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Fahr schneller du lahme Ente oder ich kotze! 'Drive faster you lame duck or I puke!'</t>
+          <t>Fahr schneller du lahme Ente oder ich kotze! ... HAHAHAHAHA! 'Drive faster you lame duck or I puke!'</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Du riechst wie eine alte Wurst! Complimenting her that she smells like an old sausage!</t>
+          <t>Du riechst wie eine alte Wurst! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Complimenting her that she smells like an old sausage!</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Das Bett ist voll mit Flöhen! Telling the hotel manager the bed is full of fleas!</t>
+          <t>Das Bett ist voll mit Flöhen! ... HAHAHAHAHA! Telling the hotel manager the bed is full of fleas!</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Mein Gehirn schmilzt hilfe! Screaming 'my brain is melting help me!' at the pharmacist</t>
+          <t>Mein Gehirn schmilzt hilfe! ... OH MY GOD!! HAHAHAHAHA! Screaming 'my brain is melting help me!' at the pharmacist</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Böser Hund beiß mich nicht! Yelling 'evil dog don't bite me!' while trembling</t>
+          <t>Böser Hund beiß mich nicht! ... HAHAHAHAHA! Yelling 'evil dog don't bite me!' while trembling</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Tais-toi américain ton accent me donne la nausée! Shouting 'Shut up American, your accent makes me vomit!'</t>
+          <t>Tais-toi américain ton accent me donne la nausée! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Shouting 'Shut up American, your accent makes me vomit!'</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Met ta baguette dans mes fesses! Asking the baker to shove his baguette up your butt!</t>
+          <t>Met ta baguette dans mes fesses! ... HAHAHAHAHA! EWWWW! Asking the baker to shove his baguette up your butt!</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Ce jus de pisse est passable! Telling the sommelier his wine tastes like passable urine!</t>
+          <t>Ce jus de pisse est passable! ... OH MY GOD!! HAHAHAHAHA! Telling the sommelier his wine tastes like passable urine!</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Lèche ma langue comme un crapaud! Asking her to lick your tongue like a toad!</t>
+          <t>Lèche ma langue comme un crapaud! ... HAHAHAHAHA! EWWWW! Asking her to lick your tongue like a toad!</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Avance connard je suis en retard! Calling the Parisian taxi driver an asshole for being slow!</t>
+          <t>Avance connard je suis en retard! ... OH MY GOD!! HAHAHAHAHA! Calling the Parisian taxi driver an asshole for being slow!</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Ce torchon me fait ressembler à un sac! Calling the designer dress a dishcloth that makes you look like a sack!</t>
+          <t>Ce torchon me fait ressembler à un sac! ... HAHAHAHAHA! Calling the designer dress a dishcloth that makes you look like a sack!</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Ça sent les pieds de mon grand-père! Informing the shopkeeper it smells like your grandpa's feet!</t>
+          <t>Ça sent les pieds de mon grand-père! ... OH MY GOD!! HAHAHAHAHA! EWWWW! Informing the shopkeeper it smells like your grandpa's feet!</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Où est la grande tour en ferraille moche? Asking for the ugly iron tower!</t>
+          <t>Où est la grande tour en ferraille moche? ... HAHAHAHAHA! Asking for the ugly iron tower!</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Donne moi du chiffon sale! Asking room service for dirty rags!</t>
+          <t>Donne moi du chiffon sale! ... OH MY GOD!! HAHAHAHAHA! Asking room service for dirty rags!</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Je t'aime mon petit boudin gras! Calling your lover a fat little blood sausage!</t>
+          <t>Je t'aime mon petit boudin gras! ... HAHAHAHAHA! EWWWW! Calling your lover a fat little blood sausage!</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">

</xml_diff>